<commit_message>
Fixed alphabetization issue for variable input
</commit_message>
<xml_diff>
--- a/2_summary_config.xlsx
+++ b/2_summary_config.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hpcdelaware-my.sharepoint.com/personal/rdietz_housingalliancede_org/Documents/Desktop/Capstone/2_summary_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hpcdelaware-my.sharepoint.com/personal/rdietz_housingalliancede_org/Documents/Desktop/Capstone/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="441" documentId="8_{58011C8A-6EEF-43E5-BA14-5EE579FB3F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD8DF8A0-0E32-4CD0-8B96-2585530A2C46}"/>
@@ -798,7 +798,7 @@
       </c>
       <c r="P2" s="3">
         <f ca="1">TODAY()</f>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q2" s="4" t="s">
         <v>18</v>
@@ -855,7 +855,7 @@
       </c>
       <c r="P3" s="3">
         <f t="shared" ref="P3:P6" ca="1" si="0">TODAY()</f>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q3" s="4" t="s">
         <v>18</v>
@@ -912,7 +912,7 @@
       </c>
       <c r="P4" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q4" s="4" t="s">
         <v>18</v>
@@ -969,7 +969,7 @@
       </c>
       <c r="P5" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q5" s="4" t="s">
         <v>18</v>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="P6" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q6" s="4" t="s">
         <v>18</v>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="P7" s="3">
         <f t="shared" ref="P7:P12" ca="1" si="1">TODAY()</f>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q7" s="4" t="s">
         <v>19</v>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="P8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q8" s="4" t="s">
         <v>20</v>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="P9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q9" s="4" t="s">
         <v>23</v>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="P10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q10" s="4" t="s">
         <v>75</v>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="P11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q11" s="4" t="s">
         <v>21</v>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="P12" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="Q12" s="4" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
fixed mixed up employment: yes and employment: no
</commit_message>
<xml_diff>
--- a/2_summary_config.xlsx
+++ b/2_summary_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hpcdelaware-my.sharepoint.com/personal/rdietz_housingalliancede_org/Documents/Desktop/Capstone/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="441" documentId="8_{58011C8A-6EEF-43E5-BA14-5EE579FB3F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD8DF8A0-0E32-4CD0-8B96-2585530A2C46}"/>
+  <xr:revisionPtr revIDLastSave="442" documentId="8_{58011C8A-6EEF-43E5-BA14-5EE579FB3F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C4F4945-E2F6-4E44-862F-85D1CD8DDA67}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15840" xr2:uid="{FD7CE67F-589C-466B-B2BE-149863F20830}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{FD7CE67F-589C-466B-B2BE-149863F20830}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="74">
   <si>
     <t>geometry</t>
   </si>
@@ -110,9 +110,6 @@
     <t>https://opendataphilly.org/datasets/philadelphia-vital-statistics-natality-births/</t>
   </si>
   <si>
-    <t>https://opendataphilly.org/datasets/philadelphia-properties-and-assessment-history/</t>
-  </si>
-  <si>
     <t>Zillow Home Value Index (ZHVI) represents the “typical” home value for a region. It’s calculated as a weighted average of the middle third of homes in a given region. When referring to the ZHVI dollar amount, it should be designated as the “typical home value for the region.” It is NOT the “median home value.”</t>
   </si>
   <si>
@@ -125,18 +122,12 @@
     <t>The Eviction Lab is a research organization dedicated to studying the prevalence, causes, and consequences of eviction. The database it has built represents the largest accumulation of U.S. court records related to eviction ever compiled.</t>
   </si>
   <si>
-    <t>Property characteristic and assessment history from the Office of Property Assessment for all properties in Philadelphia. </t>
-  </si>
-  <si>
     <t>Vital Statistics tables that contain aggregate metrics on the natality (births) of Philadelphia residents. Included in these datasets are natality metrics by planning district.</t>
   </si>
   <si>
     <t>summary_ACS_Demographics</t>
   </si>
   <si>
-    <t>summary_Philadelphia_Properties</t>
-  </si>
-  <si>
     <t>summary_Vital_Statistics_Natality</t>
   </si>
   <si>
@@ -159,9 +150,6 @@
   </si>
   <si>
     <t>total_crimes;Aggravated_Assault_No_Firearm;Disorderly_Conduct;Other_Assaults;Thefts;Vandalism..fslash..Criminal_Mischief;Theft_from_Vehicle;Fraud;All_Other_Offenses;DRIVING_UNDER_THE_INFLUENCE;Narcotic_..fslash.._Drug_Law_Violations;Burglary_Residential;Robbery_Firearm;Burglary_Non..hyphen..Residential;Motor_Vehicle_Theft;Other_Sex_Offenses_..oparen..Not_Commercialized..cparen..;Robbery_No_Firearm;Embezzlement;Aggravated_Assault_Firearm;Arson;Forgery_and_Counterfeiting;Rape;Weapon_Violations;Liquor_Law_Violations;Public_Drunkenness;Offenses_Against_Family_and_Children;Vagrancy..fslash..Loitering;Prostitution_and_Commercialized_Vice;Homicide_..hyphen.._Criminal;Gambling_Violations;Receiving_Stolen_Property;Homicide_..hyphen.._Justifiable;Part_1_Violent;Part_1_Property;Homicide_..hyphen.._Gross_Negligence</t>
-  </si>
-  <si>
-    <t>total_properties;VACANT_LAND;SINGLE_FAMILY;APARTMENTS__..greaterthan.._4_UNITS;COMMERCIAL;GARAGE_..hyphen.._COMMERCIAL;GARAGE_..hyphen.._RESIDENTIAL;HOTEL;INDUSTRIAL;MIXED_USE;MULTI_FAMILY;OFFICES;VACANT_LAND_..hyphen.._NON..hyphen..RESIDENTIAL;VACANT_LAND_..hyphen.._RESIDENTIAL;RETAIL;SPECIAL_PURPOSE</t>
   </si>
   <si>
     <t>derived_col_1</t>
@@ -674,7 +662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A518ED5D-BDC9-4209-83AA-1797F8E97236}">
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29" style="2" customWidth="1"/>
@@ -711,34 +699,34 @@
         <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>15</v>
@@ -752,10 +740,10 @@
     </row>
     <row r="2" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>14</v>
@@ -767,10 +755,10 @@
         <v>6</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>4</v>
@@ -798,21 +786,21 @@
       </c>
       <c r="P2" s="3">
         <f ca="1">TODAY()</f>
-        <v>46205</v>
+        <v>46211</v>
       </c>
       <c r="Q2" s="4" t="s">
         <v>18</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>14</v>
@@ -824,10 +812,10 @@
         <v>6</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>4</v>
@@ -855,21 +843,21 @@
       </c>
       <c r="P3" s="3">
         <f t="shared" ref="P3:P6" ca="1" si="0">TODAY()</f>
-        <v>46205</v>
+        <v>46211</v>
       </c>
       <c r="Q3" s="4" t="s">
         <v>18</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>14</v>
@@ -881,28 +869,28 @@
         <v>6</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="H4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="J4" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>62</v>
-      </c>
       <c r="M4" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="N4" s="2" t="s">
         <v>4</v>
@@ -912,21 +900,21 @@
       </c>
       <c r="P4" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>46205</v>
+        <v>46211</v>
       </c>
       <c r="Q4" s="4" t="s">
         <v>18</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>14</v>
@@ -938,16 +926,16 @@
         <v>6</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>4</v>
@@ -969,21 +957,21 @@
       </c>
       <c r="P5" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>46205</v>
+        <v>46211</v>
       </c>
       <c r="Q5" s="4" t="s">
         <v>18</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>14</v>
@@ -995,10 +983,10 @@
         <v>6</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>4</v>
@@ -1026,21 +1014,21 @@
       </c>
       <c r="P6" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>46205</v>
+        <v>46211</v>
       </c>
       <c r="Q6" s="4" t="s">
         <v>18</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>12</v>
@@ -1052,16 +1040,16 @@
         <v>6</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>4</v>
@@ -1082,22 +1070,22 @@
         <v>4</v>
       </c>
       <c r="P7" s="3">
-        <f t="shared" ref="P7:P12" ca="1" si="1">TODAY()</f>
-        <v>46205</v>
+        <f t="shared" ref="P7:P11" ca="1" si="1">TODAY()</f>
+        <v>46211</v>
       </c>
       <c r="Q7" s="4" t="s">
         <v>19</v>
       </c>
       <c r="R7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>13</v>
@@ -1109,10 +1097,10 @@
         <v>6</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>4</v>
@@ -1140,21 +1128,21 @@
       </c>
       <c r="P8" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46205</v>
+        <v>46211</v>
       </c>
       <c r="Q8" s="4" t="s">
         <v>20</v>
       </c>
       <c r="R8" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="63" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>12</v>
@@ -1166,10 +1154,10 @@
         <v>6</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>4</v>
@@ -1197,30 +1185,30 @@
       </c>
       <c r="P9" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46205</v>
+        <v>46211</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>28</v>
+        <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="63" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>77</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>4</v>
@@ -1254,30 +1242,30 @@
       </c>
       <c r="P10" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46205</v>
+        <v>46211</v>
       </c>
       <c r="Q10" s="4" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>76</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>4</v>
@@ -1311,84 +1299,26 @@
       </c>
       <c r="P11" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>46205</v>
+        <v>46211</v>
       </c>
       <c r="Q11" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R11" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="O12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="P12" s="3">
-        <f t="shared" ca="1" si="1"/>
-        <v>46205</v>
-      </c>
-      <c r="Q12" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="R12" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="Q8" r:id="rId1" xr:uid="{F3241516-93C2-476B-A81F-7FFFF2AF179B}"/>
-    <hyperlink ref="Q9" r:id="rId2" xr:uid="{D4CF80BE-CF46-4BD8-AB4D-B036F7D7EEAE}"/>
-    <hyperlink ref="Q11" r:id="rId3" xr:uid="{6B3B6708-D8F9-453C-A009-828C3ABE99C1}"/>
-    <hyperlink ref="Q12" r:id="rId4" xr:uid="{E09672A6-BA23-4330-B2EE-85E20368D50D}"/>
-    <hyperlink ref="Q7" r:id="rId5" xr:uid="{EEF0243D-8982-4C49-A21D-2E9EA12B1F8B}"/>
-    <hyperlink ref="Q2" r:id="rId6" xr:uid="{36B120BD-6E09-427B-BE9F-98CCD4C19F7C}"/>
-    <hyperlink ref="Q3" r:id="rId7" xr:uid="{4F4C41A0-9295-4A06-9B51-E2FB79D068F3}"/>
-    <hyperlink ref="Q4" r:id="rId8" xr:uid="{B3F42116-BDE0-438B-A08F-FB3A88A2AB88}"/>
-    <hyperlink ref="Q5" r:id="rId9" xr:uid="{D35ADD60-7D84-4816-B551-821D6A601CAA}"/>
-    <hyperlink ref="Q6" r:id="rId10" xr:uid="{C914AFB7-CCC5-4AA6-8B03-58A37EAA7A11}"/>
+    <hyperlink ref="Q10" r:id="rId2" xr:uid="{6B3B6708-D8F9-453C-A009-828C3ABE99C1}"/>
+    <hyperlink ref="Q11" r:id="rId3" xr:uid="{E09672A6-BA23-4330-B2EE-85E20368D50D}"/>
+    <hyperlink ref="Q7" r:id="rId4" xr:uid="{EEF0243D-8982-4C49-A21D-2E9EA12B1F8B}"/>
+    <hyperlink ref="Q2" r:id="rId5" xr:uid="{36B120BD-6E09-427B-BE9F-98CCD4C19F7C}"/>
+    <hyperlink ref="Q3" r:id="rId6" xr:uid="{4F4C41A0-9295-4A06-9B51-E2FB79D068F3}"/>
+    <hyperlink ref="Q4" r:id="rId7" xr:uid="{B3F42116-BDE0-438B-A08F-FB3A88A2AB88}"/>
+    <hyperlink ref="Q5" r:id="rId8" xr:uid="{D35ADD60-7D84-4816-B551-821D6A601CAA}"/>
+    <hyperlink ref="Q6" r:id="rId9" xr:uid="{C914AFB7-CCC5-4AA6-8B03-58A37EAA7A11}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>